<commit_message>
docs(cards): sync latest card design table
</commit_message>
<xml_diff>
--- a/Exusiai_Cardlist.xlsx
+++ b/Exusiai_Cardlist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project_spare\sts2_mod\AK_Exusiai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702A000B-E961-4489-B029-8243C953AA25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D670E3DD-53BF-4EFE-8691-FAC14F2824DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -400,9 +400,6 @@
     <t>Penguin Freight</t>
   </si>
   <si>
-    <t>所有手牌获得快递3</t>
-  </si>
-  <si>
     <t>乐观天性</t>
   </si>
   <si>
@@ -1034,6 +1031,10 @@
   </si>
   <si>
     <t>Looking Back</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有手牌获得快递3，消耗</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -1969,7 +1970,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>12</v>
@@ -1984,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="52" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>9</v>
@@ -1998,7 +1999,7 @@
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>12</v>
@@ -2013,7 +2014,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="52" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>9</v>
@@ -2027,7 +2028,7 @@
         <v>24</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>12</v>
@@ -2042,7 +2043,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="52" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>9</v>
@@ -2056,7 +2057,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>12</v>
@@ -2071,7 +2072,7 @@
         <v>1</v>
       </c>
       <c r="H8" s="52" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>9</v>
@@ -2085,7 +2086,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="53" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>12</v>
@@ -2114,7 +2115,7 @@
         <v>29</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>12</v>
@@ -2143,7 +2144,7 @@
         <v>31</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>12</v>
@@ -2172,7 +2173,7 @@
         <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>12</v>
@@ -2201,7 +2202,7 @@
         <v>36</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>12</v>
@@ -2230,7 +2231,7 @@
         <v>39</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>12</v>
@@ -2259,7 +2260,7 @@
         <v>41</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>18</v>
@@ -2288,7 +2289,7 @@
         <v>43</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>18</v>
@@ -2317,7 +2318,7 @@
         <v>45</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>18</v>
@@ -2346,7 +2347,7 @@
         <v>47</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>18</v>
@@ -2375,7 +2376,7 @@
         <v>49</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>18</v>
@@ -2404,7 +2405,7 @@
         <v>52</v>
       </c>
       <c r="C20" s="53" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>18</v>
@@ -2433,7 +2434,7 @@
         <v>54</v>
       </c>
       <c r="C21" s="53" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>18</v>
@@ -2462,7 +2463,7 @@
         <v>56</v>
       </c>
       <c r="C22" s="53" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>18</v>
@@ -2491,7 +2492,7 @@
         <v>58</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>18</v>
@@ -2506,7 +2507,7 @@
         <v>2</v>
       </c>
       <c r="H23" s="52" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>9</v>
@@ -2520,7 +2521,7 @@
         <v>59</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>18</v>
@@ -2535,7 +2536,7 @@
         <v>3</v>
       </c>
       <c r="H24" s="52" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>9</v>
@@ -3304,8 +3305,8 @@
       <c r="G49" s="2">
         <v>2</v>
       </c>
-      <c r="H49" s="4" t="s">
-        <v>121</v>
+      <c r="H49" s="52" t="s">
+        <v>328</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>9</v>
@@ -3316,7 +3317,7 @@
         <v>45</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>18</v>
@@ -3331,10 +3332,10 @@
         <v>3</v>
       </c>
       <c r="H50" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="I50" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="I50" s="4" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:26">
@@ -3342,7 +3343,7 @@
         <v>46</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>9</v>
@@ -3357,10 +3358,10 @@
         <v>61</v>
       </c>
       <c r="G51" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H51" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="H51" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>9</v>
@@ -3371,13 +3372,13 @@
         <v>47</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>13</v>
@@ -3389,7 +3390,7 @@
         <v>1</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>9</v>
@@ -3400,13 +3401,13 @@
         <v>48</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C53" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="15" t="s">
-        <v>132</v>
-      </c>
       <c r="D53" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>13</v>
@@ -3418,7 +3419,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>9</v>
@@ -3429,13 +3430,13 @@
         <v>49</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C54" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="C54" s="15" t="s">
-        <v>135</v>
-      </c>
       <c r="D54" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>13</v>
@@ -3447,7 +3448,7 @@
         <v>1</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>9</v>
@@ -3458,13 +3459,13 @@
         <v>50</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>13</v>
@@ -3476,7 +3477,7 @@
         <v>1</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>9</v>
@@ -3487,13 +3488,13 @@
         <v>51</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>13</v>
@@ -3505,7 +3506,7 @@
         <v>1</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>9</v>
@@ -3516,10 +3517,10 @@
         <v>52</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E57" s="14" t="s">
         <v>13</v>
@@ -3531,7 +3532,7 @@
         <v>1</v>
       </c>
       <c r="H57" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="58" spans="1:26">
@@ -3539,13 +3540,13 @@
         <v>53</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>13</v>
@@ -3557,7 +3558,7 @@
         <v>1</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>9</v>
@@ -3568,13 +3569,13 @@
         <v>54</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>13</v>
@@ -3586,7 +3587,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:26">
@@ -3594,13 +3595,13 @@
         <v>55</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="D60" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>13</v>
@@ -3612,7 +3613,7 @@
         <v>2</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>9</v>
@@ -3703,7 +3704,7 @@
         <v>56</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>9</v>
@@ -3715,13 +3716,13 @@
         <v>13</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G62" s="2">
         <v>0</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>9</v>
@@ -3732,7 +3733,7 @@
         <v>57</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>9</v>
@@ -3744,13 +3745,13 @@
         <v>13</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G63" s="2">
         <v>1</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>9</v>
@@ -3761,7 +3762,7 @@
         <v>58</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>9</v>
@@ -3773,13 +3774,13 @@
         <v>13</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G64" s="2">
         <v>2</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>9</v>
@@ -3790,10 +3791,10 @@
         <v>59</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>12</v>
@@ -3802,13 +3803,13 @@
         <v>13</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G65" s="2">
         <v>3</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>9</v>
@@ -3819,7 +3820,7 @@
         <v>60</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>9</v>
@@ -3831,13 +3832,13 @@
         <v>13</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G66" s="2">
         <v>3</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>9</v>
@@ -3848,10 +3849,10 @@
         <v>61</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>12</v>
@@ -3860,13 +3861,13 @@
         <v>13</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G67" s="2">
         <v>5</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>9</v>
@@ -3877,10 +3878,10 @@
         <v>62</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
@@ -3889,13 +3890,13 @@
         <v>13</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G68" s="2">
         <v>6</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>9</v>
@@ -3906,7 +3907,7 @@
         <v>63</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D69" s="14" t="s">
         <v>18</v>
@@ -3915,16 +3916,16 @@
         <v>13</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G69" s="2">
         <v>0</v>
       </c>
       <c r="H69" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="I69" s="13" t="s">
         <v>169</v>
-      </c>
-      <c r="I69" s="13" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3932,7 +3933,7 @@
         <v>64</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>9</v>
@@ -3944,13 +3945,13 @@
         <v>13</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G70" s="2">
         <v>0</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>79</v>
@@ -3961,7 +3962,7 @@
         <v>65</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>18</v>
@@ -3970,13 +3971,13 @@
         <v>13</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G71" s="2">
         <v>0</v>
       </c>
       <c r="H71" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>9</v>
@@ -3987,7 +3988,7 @@
         <v>66</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>9</v>
@@ -3999,13 +4000,13 @@
         <v>13</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G72" s="2">
         <v>0</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>9</v>
@@ -4016,7 +4017,7 @@
         <v>67</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>9</v>
@@ -4028,13 +4029,13 @@
         <v>13</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G73" s="2">
         <v>1</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>9</v>
@@ -4045,10 +4046,10 @@
         <v>68</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>18</v>
@@ -4057,13 +4058,13 @@
         <v>13</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G74" s="2">
         <v>5</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>9</v>
@@ -4074,7 +4075,7 @@
         <v>69</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>9</v>
@@ -4086,13 +4087,13 @@
         <v>13</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G75" s="2">
         <v>6</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>9</v>
@@ -4103,7 +4104,7 @@
         <v>70</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>9</v>
@@ -4115,13 +4116,13 @@
         <v>13</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G76" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H76" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>9</v>
@@ -4132,25 +4133,25 @@
         <v>71</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D77" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G77" s="2">
         <v>0</v>
       </c>
       <c r="H77" s="21" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>9</v>
@@ -4161,28 +4162,28 @@
         <v>72</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G78" s="2">
         <v>0</v>
       </c>
       <c r="H78" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="I78" s="4" t="s">
         <v>189</v>
-      </c>
-      <c r="I78" s="4" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -4190,25 +4191,25 @@
         <v>73</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G79" s="2">
         <v>1</v>
       </c>
       <c r="H79" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>9</v>
@@ -4219,22 +4220,22 @@
         <v>74</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D80" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E80" s="14" t="s">
         <v>13</v>
       </c>
       <c r="F80" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G80" s="2">
         <v>1</v>
       </c>
       <c r="H80" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>9</v>
@@ -4245,25 +4246,25 @@
         <v>75</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G81" s="2">
         <v>1</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="82" spans="1:26">
@@ -4271,25 +4272,25 @@
         <v>76</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C82" s="2" t="s">
-        <v>198</v>
-      </c>
       <c r="D82" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G82" s="2">
         <v>1</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>9</v>
@@ -4300,25 +4301,25 @@
         <v>77</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C83" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="D83" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G83" s="2">
         <v>2</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>9</v>
@@ -4329,28 +4330,28 @@
         <v>78</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G84" s="2">
         <v>3</v>
       </c>
       <c r="H84" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="I84" s="13" t="s">
         <v>204</v>
-      </c>
-      <c r="I84" s="13" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="85" spans="1:26">
@@ -4358,25 +4359,25 @@
         <v>79</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G85" s="2">
         <v>3</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>9</v>
@@ -4387,25 +4388,25 @@
         <v>80</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G86" s="2">
         <v>4</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>9</v>
@@ -4496,28 +4497,28 @@
         <v>81</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>211</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E88" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F88" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G88" s="2">
         <v>0</v>
       </c>
       <c r="H88" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="I88" s="24" t="s">
         <v>214</v>
-      </c>
-      <c r="I88" s="24" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="89" spans="1:26">
@@ -4525,28 +4526,28 @@
         <v>82</v>
       </c>
       <c r="B89" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E89" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F89" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G89" s="2">
         <v>0</v>
       </c>
       <c r="H89" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="I89" s="24" t="s">
         <v>218</v>
-      </c>
-      <c r="I89" s="24" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="90" spans="1:26">
@@ -4554,28 +4555,28 @@
         <v>83</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>221</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E90" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F90" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G90" s="2">
         <v>0</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I90" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="91" spans="1:26">
@@ -4583,28 +4584,28 @@
         <v>84</v>
       </c>
       <c r="B91" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E91" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F91" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G91" s="2">
         <v>0</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I91" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="92" spans="1:26">
@@ -4612,28 +4613,28 @@
         <v>85</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>227</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E92" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F92" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F92" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G92" s="2">
         <v>1</v>
       </c>
       <c r="H92" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="I92" s="24" t="s">
         <v>228</v>
-      </c>
-      <c r="I92" s="24" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="93" spans="1:26">
@@ -4641,28 +4642,28 @@
         <v>86</v>
       </c>
       <c r="B93" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>231</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E93" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F93" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G93" s="2">
         <v>0</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I93" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="94" spans="1:26">
@@ -4670,28 +4671,28 @@
         <v>87</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>234</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E94" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F94" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G94" s="2">
         <v>0</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I94" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J94" s="3" t="s">
         <v>9</v>
@@ -4750,28 +4751,28 @@
         <v>88</v>
       </c>
       <c r="B95" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E95" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F95" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F95" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G95" s="2">
         <v>0</v>
       </c>
       <c r="H95" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I95" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J95" s="3" t="s">
         <v>9</v>
@@ -4830,7 +4831,7 @@
         <v>89</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>9</v>
@@ -4839,19 +4840,19 @@
         <v>18</v>
       </c>
       <c r="E96" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F96" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="G96" s="2">
         <v>0</v>
       </c>
       <c r="H96" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="I96" s="24" t="s">
         <v>240</v>
-      </c>
-      <c r="I96" s="24" t="s">
-        <v>241</v>
       </c>
       <c r="J96" s="3" t="s">
         <v>9</v>
@@ -4910,25 +4911,25 @@
         <v>90</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C97" s="53" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D97" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E97" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F97" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="F97" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="G97" s="2">
         <v>0</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J97" s="3" t="s">
         <v>9</v>
@@ -4987,7 +4988,7 @@
         <v>91</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>9</v>
@@ -4996,16 +4997,16 @@
         <v>18</v>
       </c>
       <c r="E98" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F98" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="G98" s="2">
         <v>1</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I98" s="4" t="s">
         <v>9</v>
@@ -5067,7 +5068,7 @@
         <v>92</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>9</v>
@@ -5076,16 +5077,16 @@
         <v>18</v>
       </c>
       <c r="E99" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F99" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="F99" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="G99" s="2">
         <v>1</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I99" s="24" t="s">
         <v>9</v>
@@ -5147,7 +5148,7 @@
         <v>93</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>9</v>
@@ -5156,16 +5157,16 @@
         <v>18</v>
       </c>
       <c r="E100" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F100" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="F100" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="G100" s="2">
         <v>0</v>
       </c>
       <c r="H100" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I100" s="4" t="s">
         <v>9</v>
@@ -5176,10 +5177,10 @@
         <v>94</v>
       </c>
       <c r="B102" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="C102" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="D102" s="14" t="s">
         <v>12</v>
@@ -5188,13 +5189,13 @@
         <v>13</v>
       </c>
       <c r="F102" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G102" s="2">
         <v>1</v>
       </c>
       <c r="H102" s="13" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I102" s="13" t="s">
         <v>10</v>
@@ -5205,25 +5206,25 @@
         <v>95</v>
       </c>
       <c r="B103" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="C103" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="C103" s="14" t="s">
-        <v>255</v>
-      </c>
       <c r="D103" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G103" s="2">
         <v>1</v>
       </c>
       <c r="H103" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="104" spans="1:26">
@@ -5777,19 +5778,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="D1" s="14" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>260</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -5803,19 +5804,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>9</v>
@@ -5826,19 +5827,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>266</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>9</v>
@@ -5867,19 +5868,19 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="B1" s="26" t="s">
         <v>267</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>268</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>269</v>
       </c>
       <c r="D1" s="26" t="s">
         <v>8</v>
       </c>
       <c r="F1" s="28" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G1" s="29" t="s">
         <v>22</v>
@@ -5888,21 +5889,21 @@
         <v>61</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J1" s="31" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="32" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="C2" s="34" t="s">
         <v>273</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>274</v>
       </c>
       <c r="D2" s="33" t="s">
         <v>9</v>
@@ -5929,13 +5930,13 @@
     </row>
     <row r="3" spans="1:10" ht="33">
       <c r="A3" s="39" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D3" s="33" t="s">
         <v>9</v>
@@ -5962,19 +5963,19 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="39" t="s">
+        <v>275</v>
+      </c>
+      <c r="B4" s="40" t="s">
         <v>276</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="C4" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="D4" s="33" t="s">
         <v>277</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>274</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>278</v>
-      </c>
       <c r="F4" s="35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G4" s="36">
         <f>COUNTIFS(工作表1!$D:$D,$F4,工作表1!$F:$F,G$1,工作表1!$G:$G,"&lt;&gt;",工作表1!$H:$H,"&lt;&gt;",工作表1!$F:$F,"&lt;&gt;衍生")</f>
@@ -5995,19 +5996,19 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="B5" s="40" t="s">
         <v>279</v>
       </c>
-      <c r="B5" s="40" t="s">
-        <v>280</v>
-      </c>
       <c r="C5" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D5" s="33" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="42" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G5" s="43">
         <f>SUM(G2:G4)</f>
@@ -6028,13 +6029,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="39" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B6" s="46" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D6" s="33" t="s">
         <v>9</v>
@@ -6042,146 +6043,146 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="39" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B7" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>273</v>
+      </c>
+      <c r="D7" s="33" t="s">
         <v>282</v>
-      </c>
-      <c r="C7" s="41" t="s">
-        <v>274</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="B8" s="46" t="s">
         <v>284</v>
       </c>
-      <c r="B8" s="46" t="s">
-        <v>285</v>
-      </c>
       <c r="C8" s="34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B9" s="46" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="49.5">
       <c r="A10" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B10" s="46" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B11" s="46" t="s">
+        <v>287</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" s="46" t="s">
         <v>288</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>274</v>
-      </c>
-      <c r="D11" s="46" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B12" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="C12" s="34" t="s">
         <v>290</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="D12" s="46" t="s">
         <v>291</v>
-      </c>
-      <c r="D12" s="46" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B13" s="46" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="39" t="s">
+        <v>293</v>
+      </c>
+      <c r="B14" s="46" t="s">
         <v>294</v>
       </c>
-      <c r="B14" s="46" t="s">
-        <v>295</v>
-      </c>
       <c r="C14" s="34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="33">
       <c r="A15" s="32" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B15" s="40" t="s">
+        <v>295</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="D15" s="46" t="s">
         <v>296</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>274</v>
-      </c>
-      <c r="D15" s="46" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="39" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B16" s="46" t="s">
+        <v>297</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="D16" s="46" t="s">
         <v>298</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>274</v>
-      </c>
-      <c r="D16" s="46" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="39" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B17" s="46" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="39" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>